<commit_message>
1st changes after DB Referesh Oct 30 2023
</commit_message>
<xml_diff>
--- a/TestData/TMTI0055029_VerifyInternalDealTeamSpecialtyRoleIncreasedLimitForCFLOBOpportunityEngagement.xlsx
+++ b/TestData/TMTI0055029_VerifyInternalDealTeamSpecialtyRoleIncreasedLimitForCFLOBOpportunityEngagement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0808CB8E-5B2A-48F5-979E-1ED8415BCCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E86F88D-30B6-4FAC-9772-7996F86E294C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14640" activeTab="5" xr2:uid="{2C05E2F5-3DB9-4FD8-8E59-14E5CD867A79}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{2C05E2F5-3DB9-4FD8-8E59-14E5CD867A79}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -723,9 +723,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D1A1FE9-CADD-4FD6-8E73-186E076A589E}">
   <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,7 +817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -917,17 +917,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF1B31D-A2B0-43BC-A587-8474F3E673D9}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -940,22 +940,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58FEA5EE-1EE6-46E7-A593-CB024A1C58ED}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -968,13 +968,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F7719AF-9118-4A60-BF7F-3491DAE91C27}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -982,9 +982,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
         <v>49</v>
@@ -998,14 +998,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87197585-6EB4-40DD-9571-6763D8C561B1}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1065,147 +1065,147 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5D3C4F-7CA4-4B49-99BD-C542C86946E3}">
   <dimension ref="A1:A28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>96</v>
       </c>
@@ -1219,17 +1219,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A1A452-25F2-430A-8358-9CDC08D43509}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1242,13 +1242,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BC13775-FB7E-4A2D-845E-DF647C6681C0}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="57.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>63</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>65</v>
       </c>

</xml_diff>